<commit_message>
first try to update prices from jsons to excel
</commit_message>
<xml_diff>
--- a/data/samsung-service-prices.xlsx
+++ b/data/samsung-service-prices.xlsx
@@ -5,15 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/89fe5ae0d6b51d32/Dokumenty/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamd\Github\maro_web\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1263232-3ABA-4269-8F4C-7B1722B30230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D98B229-726E-4510-985A-5E329587C127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{7086E827-2BEE-473B-BA1A-5CAD5929993F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="galaxy-a" sheetId="1" r:id="rId1"/>
+    <sheet name="galaxy-m" sheetId="2" r:id="rId2"/>
+    <sheet name="galaxy-note" sheetId="3" r:id="rId3"/>
+    <sheet name="galaxy-s" sheetId="4" r:id="rId4"/>
+    <sheet name="galaxy-z" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,15 +39,50 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="8">
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>displej</t>
+  </si>
+  <si>
+    <t>bateria</t>
+  </si>
+  <si>
+    <t>nabijanie</t>
+  </si>
+  <si>
+    <t>tekutina</t>
+  </si>
+  <si>
+    <t>diagnostika</t>
+  </si>
+  <si>
+    <t>inyproblem</t>
+  </si>
+  <si>
+    <t>backglass</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -67,8 +106,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,9 +443,225 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68E7282C-F129-45FA-83C9-ABA740391124}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="11.85546875" customWidth="1"/>
+    <col min="19" max="19" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B9B2FEE-3C95-42A1-8584-CD1B534DDFB4}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" customWidth="1"/>
+    <col min="19" max="20" width="11.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE6E7198-150F-4C2D-871F-8E67716203E4}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF61A20-544B-4258-9AF5-8897163C8398}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6086A363-4DB7-42D2-BA8D-A020BDF26AE5}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>